<commit_message>
Updates to use new capital costs for hydro from NEXT Group, disallows new hydro from being built, updates capacity factors as discussed on About page.
</commit_message>
<xml_diff>
--- a/InputData/elec/MPCbS/Max Potential Capacity by Source.xlsx
+++ b/InputData/elec/MPCbS/Max Potential Capacity by Source.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Dropbox\NEXT Group\90. 개인 폴더\이지우\단기대응\202501 EPS 수요전망\V3\MPCbS\old\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\MPCbS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{057250BD-3CB9-4FBE-9392-1A832EAC6CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28FB656-BB7B-4EEA-B972-4F555B729A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="38">
   <si>
     <t>Source:</t>
   </si>
@@ -150,6 +150,9 @@
   <si>
     <t>KNREC</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>We limit hydro at current capacity as we do not expect more to be built.</t>
   </si>
 </sst>
 </file>
@@ -157,13 +160,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -171,7 +174,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -179,13 +182,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -193,14 +196,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -240,7 +243,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -248,8 +251,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -265,9 +268,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -305,9 +308,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -340,26 +343,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -392,26 +378,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -585,18 +554,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="60.796875" customWidth="1"/>
+    <col min="2" max="2" width="60.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -604,49 +573,54 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2">
       <c r="B4" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2">
       <c r="B5" s="3">
         <v>2020</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2">
       <c r="B6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2">
       <c r="B7" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2">
       <c r="B8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -663,15 +637,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.19921875" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -679,7 +653,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -688,7 +662,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -697,7 +671,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -706,7 +680,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -715,7 +689,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -723,7 +697,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -731,7 +705,7 @@
         <v>352000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -740,7 +714,7 @@
       </c>
       <c r="G8" s="5"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -749,7 +723,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -757,7 +731,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -765,7 +739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -774,7 +748,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -783,7 +757,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -791,7 +765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -799,7 +773,7 @@
         <v>387000</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -807,7 +781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -815,7 +789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -823,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -832,7 +806,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -841,7 +815,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -849,7 +823,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -857,7 +831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -866,7 +840,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:2">
       <c r="A24" s="7" t="s">
         <v>33</v>
       </c>
@@ -875,7 +849,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:2">
       <c r="A25" s="7" t="s">
         <v>34</v>
       </c>
@@ -897,14 +871,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="27.19921875" customWidth="1"/>
-    <col min="3" max="3" width="24.8984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -912,7 +886,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -921,7 +895,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -930,7 +904,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -939,7 +913,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -948,16 +922,15 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="6">
-        <f>Data!B6</f>
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -966,7 +939,7 @@
         <v>352000</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -975,7 +948,7 @@
         <v>2409000</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -984,7 +957,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -993,7 +966,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1002,7 +975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1011,7 +984,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1020,7 +993,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1029,7 +1002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -1038,7 +1011,7 @@
         <v>387000</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1047,7 +1020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1056,7 +1029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -1065,7 +1038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1074,7 +1047,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1083,7 +1056,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -1092,7 +1065,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -1101,7 +1074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1110,7 +1083,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:2">
       <c r="A24" s="7" t="s">
         <v>33</v>
       </c>
@@ -1119,7 +1092,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:2">
       <c r="A25" s="7" t="s">
         <v>34</v>
       </c>
@@ -1136,6 +1109,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -1279,29 +1267,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB8A1281-739A-44F7-B3AB-B77AE3020F80}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C335326-399A-4580-9714-6B4BBF76165B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9C21EDA-1272-4856-97A0-2867CE6DDD78}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9C21EDA-1272-4856-97A0-2867CE6DDD78}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C335326-399A-4580-9714-6B4BBF76165B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB8A1281-739A-44F7-B3AB-B77AE3020F80}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>